<commit_message>
Convert hero-video block to hero-image
Rename the hero-video block/parser/model to hero-image and drop the
background-video carrier (mp4). The hero now migrates as a still image
(fallback homepage_hero.png) so it previews reliably in EDS and AEM.

- blocks/hero-image/ (renamed from hero-video; CSS selectors + model id
  + component title "Hero Image" updated)
- tools/importer/parsers/hero-image.js (drops mp4 extraction + carrier anchor)
- page-templates.json + import-homepage.js reference hero-image
- rebuilt component-*.json; re-imported content/index.plain.html
- regenerated JCR (index.xml) + refreshed content package zip

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-video","cards-stats","columns-feature","columns-feature","columns-feature","cards-logos","columns-stock","carousel-news"]</t>
+    <t>["hero-image","cards-stats","columns-feature","columns-feature","columns-feature","cards-logos","columns-stock","carousel-news"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-08-12T23:20:05.202Z</t>
+    <t>2026-08-13T15:32:22.024Z</t>
   </si>
   <si>
     <t>Home | Covista</t>

</xml_diff>